<commit_message>
[add] [history] Penambahan Fitur History & Perbaikan BUG Perhitungan
</commit_message>
<xml_diff>
--- a/public/Pehitungan SMART Rekomendasi Mobil.xlsx
+++ b/public/Pehitungan SMART Rekomendasi Mobil.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trimi\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF940D48-B572-428D-9937-C3B594B16CDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A893621-733D-4993-A23D-2A801E58E768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-90" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{8A6E19D3-3902-4506-86DB-5E2E20D39654}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="21840" windowHeight="13020" xr2:uid="{8A6E19D3-3902-4506-86DB-5E2E20D39654}"/>
   </bookViews>
   <sheets>
     <sheet name="Perhitungan" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="77">
   <si>
     <t>No</t>
   </si>
@@ -166,33 +166,18 @@
     <t>capacity_machine</t>
   </si>
   <si>
-    <t>Brio</t>
-  </si>
-  <si>
-    <t>Hr-v</t>
-  </si>
-  <si>
     <t>Platinum White Pearl</t>
   </si>
   <si>
-    <t>Brv</t>
-  </si>
-  <si>
     <t>Putih</t>
   </si>
   <si>
     <t>Civic</t>
   </si>
   <si>
-    <t>Wrv</t>
-  </si>
-  <si>
     <t>City</t>
   </si>
   <si>
-    <t>Cr-v</t>
-  </si>
-  <si>
     <t>Canyon River Blue Metallic</t>
   </si>
   <si>
@@ -202,9 +187,6 @@
     <t>Accord</t>
   </si>
   <si>
-    <t>Platinum white pearl</t>
-  </si>
-  <si>
     <t>slug</t>
   </si>
   <si>
@@ -244,18 +226,6 @@
     <t>value</t>
   </si>
   <si>
-    <t>&gt; 616000000</t>
-  </si>
-  <si>
-    <t>380000000 - 540000000</t>
-  </si>
-  <si>
-    <t>285000000 - 320000000</t>
-  </si>
-  <si>
-    <t>180000000 - 253100000</t>
-  </si>
-  <si>
     <t>Pearl Gray Metallic</t>
   </si>
   <si>
@@ -269,6 +239,39 @@
   </si>
   <si>
     <t>Merah</t>
+  </si>
+  <si>
+    <t>&gt; 540000000</t>
+  </si>
+  <si>
+    <t>320000000 - 540000000</t>
+  </si>
+  <si>
+    <t>253100000 - 320000000</t>
+  </si>
+  <si>
+    <t>150000000 - 253100000</t>
+  </si>
+  <si>
+    <t>\N</t>
+  </si>
+  <si>
+    <t>Brio Satya</t>
+  </si>
+  <si>
+    <t>HR-V</t>
+  </si>
+  <si>
+    <t>BR-V</t>
+  </si>
+  <si>
+    <t>WR-V</t>
+  </si>
+  <si>
+    <t>CR-V</t>
+  </si>
+  <si>
+    <t>Brio RS</t>
   </si>
 </sst>
 </file>
@@ -425,7 +428,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -474,6 +477,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -817,11 +823,12 @@
     <col min="3" max="3" width="23.140625" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -832,7 +839,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="4">
         <v>1</v>
       </c>
@@ -843,7 +850,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="7">
         <v>2</v>
       </c>
@@ -854,7 +861,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="4">
         <v>3</v>
       </c>
@@ -865,7 +872,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="7">
         <v>4</v>
       </c>
@@ -876,12 +883,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
         <v>1</v>
       </c>
@@ -898,7 +905,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="8"/>
       <c r="C11" s="11">
         <f>35/100</f>
@@ -917,13 +924,13 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="13" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="22"/>
     </row>
-    <row r="14" spans="2:6" s="15" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:9" s="15" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="14" t="s">
         <v>13</v>
       </c>
@@ -940,177 +947,247 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="2:6" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="8" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="C15" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="12">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E15" s="12">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F15" s="12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="2:6" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I15" t="str">
+        <f>VLOOKUP(H15,'Data Mobil'!$C$2:$H$11,2)</f>
+        <v>Mobilio</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C16" s="12">
+        <v>2</v>
+      </c>
+      <c r="D16" s="12">
+        <v>4</v>
+      </c>
+      <c r="E16" s="12">
+        <v>4</v>
+      </c>
+      <c r="F16" s="12">
+        <v>1</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" t="str">
+        <f>VLOOKUP(H16,'Data Mobil'!$C$2:$H$11,2)</f>
+        <v>BR-V</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="12">
         <v>3</v>
       </c>
-      <c r="D16" s="12">
-        <v>0</v>
-      </c>
-      <c r="E16" s="12">
-        <v>0</v>
-      </c>
-      <c r="F16" s="12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17" s="12">
+      <c r="D17" s="12">
         <v>2</v>
       </c>
-      <c r="D17" s="12">
-        <v>4</v>
-      </c>
       <c r="E17" s="12">
         <v>4</v>
       </c>
       <c r="F17" s="12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I17" t="str">
+        <f>VLOOKUP(H17,'Data Mobil'!$C$2:$H$11,2)</f>
+        <v>City</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="8" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C18" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" s="12">
         <v>2</v>
       </c>
       <c r="E18" s="12">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F18" s="12">
+        <v>3</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18" t="str">
+        <f>VLOOKUP(H18,'Data Mobil'!$C$2:$H$11,2)</f>
+        <v>Brio Satya</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="12">
+        <v>1</v>
+      </c>
+      <c r="D19" s="12">
+        <v>2</v>
+      </c>
+      <c r="E19" s="12">
+        <v>1</v>
+      </c>
+      <c r="F19" s="12">
+        <v>2</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I19" t="str">
+        <f>VLOOKUP(H19,'Data Mobil'!$C$2:$H$11,2)</f>
+        <v>Brio Satya</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="12">
+        <v>2</v>
+      </c>
+      <c r="D20" s="12">
+        <v>2</v>
+      </c>
+      <c r="E20" s="12">
+        <v>1</v>
+      </c>
+      <c r="F20" s="12">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="2:6" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="8" t="s">
+      <c r="H20" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="12">
-        <v>0</v>
-      </c>
-      <c r="D19" s="12">
-        <v>0</v>
-      </c>
-      <c r="E19" s="12">
-        <v>0</v>
-      </c>
-      <c r="F19" s="12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C20" s="12">
-        <v>0</v>
-      </c>
-      <c r="D20" s="12">
-        <v>0</v>
-      </c>
-      <c r="E20" s="12">
-        <v>4</v>
-      </c>
-      <c r="F20" s="12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I20" t="str">
+        <f>VLOOKUP(H20,'Data Mobil'!$C$2:$H$11,2)</f>
+        <v>WR-V</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="12">
+        <v>4</v>
+      </c>
+      <c r="D21" s="12">
+        <v>2</v>
+      </c>
+      <c r="E21" s="12">
+        <v>4</v>
+      </c>
+      <c r="F21" s="12">
+        <v>7</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" t="str">
+        <f>VLOOKUP(H21,'Data Mobil'!$C$2:$H$11,2)</f>
+        <v>Civic</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="12">
+        <v>3</v>
+      </c>
+      <c r="D22" s="12">
+        <v>2</v>
+      </c>
+      <c r="E22" s="12">
+        <v>1</v>
+      </c>
+      <c r="F22" s="12">
+        <v>6</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" t="str">
+        <f>VLOOKUP(H22,'Data Mobil'!$C$2:$H$11,2)</f>
+        <v>HR-V</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="12">
-        <v>4</v>
-      </c>
-      <c r="D21" s="12">
-        <v>0</v>
-      </c>
-      <c r="E21" s="12">
-        <v>0</v>
-      </c>
-      <c r="F21" s="12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="12">
-        <v>1</v>
-      </c>
-      <c r="D22" s="12">
-        <v>4</v>
-      </c>
-      <c r="E22" s="12">
-        <v>4</v>
-      </c>
-      <c r="F22" s="12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="8" t="s">
+      <c r="C23" s="12">
+        <v>4</v>
+      </c>
+      <c r="D23" s="12">
+        <v>2</v>
+      </c>
+      <c r="E23" s="12">
+        <v>1</v>
+      </c>
+      <c r="F23" s="12">
+        <v>8</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I23" t="str">
+        <f>VLOOKUP(H23,'Data Mobil'!$C$2:$H$11,2)</f>
+        <v>CR-V</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="12">
-        <v>4</v>
-      </c>
-      <c r="D23" s="12">
-        <v>0</v>
-      </c>
-      <c r="E23" s="12">
-        <v>0</v>
-      </c>
-      <c r="F23" s="12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="8" t="s">
-        <v>23</v>
-      </c>
       <c r="C24" s="12">
         <v>4</v>
       </c>
       <c r="D24" s="12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E24" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" s="12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="I24" t="str">
+        <f>VLOOKUP(H24,'Data Mobil'!$C$2:$H$11,2)</f>
+        <v>Accord</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C25" s="10" t="s">
         <v>24</v>
       </c>
@@ -1124,13 +1201,13 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="22" t="s">
         <v>26</v>
       </c>
       <c r="C27" s="22"/>
     </row>
-    <row r="28" spans="2:6" s="15" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:9" s="15" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="14" t="s">
         <v>13</v>
       </c>
@@ -1147,9 +1224,10 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="2:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="8" t="s">
-        <v>14</v>
+    <row r="29" spans="2:9" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="8" t="str">
+        <f>B15</f>
+        <v>P8</v>
       </c>
       <c r="C29" s="13">
         <f>((MAX(C$15:C$24)-C15))/(MAX(C$15:C$24)-MIN(C$15:C$24))</f>
@@ -1157,204 +1235,213 @@
       </c>
       <c r="D29" s="13">
         <f>((D15-(MIN(D$15:D$24)))/((MAX(D$15:D$24))-(MIN(D$15:D$24))))*100%</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" s="13">
         <f t="shared" ref="E29:F29" si="0">((E15-(MIN(E$15:E$24)))/((MAX(E$15:E$24))-(MIN(E$15:E$24))))*100%</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" s="13">
         <f t="shared" si="0"/>
-        <v>0.16666666666666666</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="8" t="s">
-        <v>15</v>
+        <v>0.5714285714285714</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="8" t="str">
+        <f t="shared" ref="B30:B38" si="1">B16</f>
+        <v>P3</v>
       </c>
       <c r="C30" s="13">
-        <f t="shared" ref="C30:C38" si="1">((MAX(C$15:C$24)-C16))/(MAX(C$15:C$24)-MIN(C$15:C$24))</f>
-        <v>0.25</v>
+        <f t="shared" ref="C30:C38" si="2">((MAX(C$15:C$24)-C16))/(MAX(C$15:C$24)-MIN(C$15:C$24))</f>
+        <v>0.66666666666666663</v>
       </c>
       <c r="D30" s="13">
-        <f t="shared" ref="D30:F38" si="2">((D16-(MIN(D$15:D$24)))/((MAX(D$15:D$24))-(MIN(D$15:D$24))))*100%</f>
-        <v>0</v>
+        <f t="shared" ref="D30:F38" si="3">((D16-(MIN(D$15:D$24)))/((MAX(D$15:D$24))-(MIN(D$15:D$24))))*100%</f>
+        <v>1</v>
       </c>
       <c r="E30" s="13">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="F30" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>P6</v>
+      </c>
+      <c r="C31" s="13">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F30" s="13">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D31" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E31" s="13">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="F31" s="13">
+        <f t="shared" si="3"/>
+        <v>0.7142857142857143</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>P10</v>
+      </c>
+      <c r="C32" s="13">
         <f t="shared" si="2"/>
-        <v>0.83333333333333337</v>
-      </c>
-    </row>
-    <row r="31" spans="2:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C31" s="13">
+        <v>1</v>
+      </c>
+      <c r="D32" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E32" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="F32" s="13">
+        <f t="shared" si="3"/>
+        <v>0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="8" t="str">
         <f t="shared" si="1"/>
-        <v>0.5</v>
-      </c>
-      <c r="D31" s="13">
+        <v>P10</v>
+      </c>
+      <c r="C33" s="13">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="E31" s="13">
+      <c r="D33" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E33" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="F33" s="13">
+        <f t="shared" si="3"/>
+        <v>0.14285714285714285</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>P5</v>
+      </c>
+      <c r="C34" s="13">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="F31" s="13">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D34" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E34" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="F34" s="13">
+        <f t="shared" si="3"/>
+        <v>0.7142857142857143</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>P4</v>
+      </c>
+      <c r="C35" s="13">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="2:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C32" s="13">
+      <c r="D35" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E35" s="13">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="F35" s="13">
+        <f t="shared" si="3"/>
+        <v>0.8571428571428571</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="8" t="str">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D32" s="13">
+        <v>P2</v>
+      </c>
+      <c r="C36" s="13">
         <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="E32" s="13">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D36" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E36" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="F36" s="13">
+        <f t="shared" si="3"/>
+        <v>0.7142857142857143</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>P7</v>
+      </c>
+      <c r="C37" s="13">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="F32" s="13">
+        <v>0</v>
+      </c>
+      <c r="D37" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E37" s="13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="F37" s="13">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>P9</v>
+      </c>
+      <c r="C38" s="13">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="2:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C33" s="13">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D33" s="13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E33" s="13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F33" s="13">
-        <f t="shared" si="2"/>
-        <v>0.83333333333333337</v>
-      </c>
-    </row>
-    <row r="34" spans="2:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C34" s="13">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D34" s="13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E34" s="13">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="F34" s="13">
-        <f t="shared" si="2"/>
-        <v>0.83333333333333337</v>
-      </c>
-    </row>
-    <row r="35" spans="2:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C35" s="13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="D35" s="13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E35" s="13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F35" s="13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="2:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C36" s="13">
-        <f t="shared" si="1"/>
-        <v>0.75</v>
-      </c>
-      <c r="D36" s="13">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="E36" s="13">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="F36" s="13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="2:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C37" s="13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="D37" s="13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E37" s="13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F37" s="13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="2:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C38" s="13">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="D38" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="E38" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F38" s="13">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1387,292 +1474,302 @@
       </c>
     </row>
     <row r="42" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="8" t="s">
-        <v>22</v>
+      <c r="B42" s="8" t="str">
+        <f>B15</f>
+        <v>P8</v>
       </c>
       <c r="C42" s="17">
-        <f t="shared" ref="C42:F51" si="3">C29*C$11</f>
+        <f t="shared" ref="C42:F51" si="4">C29*C$11</f>
         <v>0.35</v>
       </c>
       <c r="D42" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>0.3</v>
       </c>
       <c r="E42" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>0.15</v>
       </c>
       <c r="F42" s="17">
-        <f t="shared" si="3"/>
-        <v>3.3333333333333333E-2</v>
+        <f t="shared" si="4"/>
+        <v>0.11428571428571428</v>
       </c>
       <c r="G42" s="18">
-        <f t="shared" ref="G42:G51" si="4">SUM(C42:F42)</f>
-        <v>0.3833333333333333</v>
-      </c>
-      <c r="H42" s="12">
-        <f t="shared" ref="H42:H51" si="5">RANK(G42,$G$42:$G$51,0)+COUNTIF($G$42:$G$51,G42)-1</f>
+        <f t="shared" ref="G42:G51" si="5">SUM(C42:F42)</f>
+        <v>0.91428571428571426</v>
+      </c>
+      <c r="H42" s="23">
+        <f>RANK(G42,$G$42:$G$51,0)+COUNTIF($G$42:G42,G42)-1</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="8" t="str">
+        <f t="shared" ref="B43:B51" si="6">B16</f>
+        <v>P3</v>
+      </c>
+      <c r="C43" s="17">
+        <f t="shared" si="4"/>
+        <v>0.23333333333333331</v>
+      </c>
+      <c r="D43" s="17">
+        <f t="shared" si="4"/>
+        <v>0.3</v>
+      </c>
+      <c r="E43" s="17">
+        <f t="shared" si="4"/>
+        <v>0.15</v>
+      </c>
+      <c r="F43" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="G43" s="18">
+        <f t="shared" si="5"/>
+        <v>0.68333333333333335</v>
+      </c>
+      <c r="H43" s="23">
+        <f>RANK(G43,$G$42:$G$51,0)+COUNTIF($G$42:G43,G43)-1</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B44" s="8" t="str">
+        <f t="shared" si="6"/>
+        <v>P6</v>
+      </c>
+      <c r="C44" s="17">
+        <f t="shared" si="4"/>
+        <v>0.11666666666666665</v>
+      </c>
+      <c r="D44" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E44" s="17">
+        <f t="shared" si="4"/>
+        <v>0.15</v>
+      </c>
+      <c r="F44" s="17">
+        <f t="shared" si="4"/>
+        <v>0.14285714285714288</v>
+      </c>
+      <c r="G44" s="18">
+        <f t="shared" si="5"/>
+        <v>0.40952380952380951</v>
+      </c>
+      <c r="H44" s="23">
+        <f>RANK(G44,$G$42:$G$51,0)+COUNTIF($G$42:G44,G44)-1</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B45" s="8" t="str">
+        <f t="shared" si="6"/>
+        <v>P10</v>
+      </c>
+      <c r="C45" s="17">
+        <f t="shared" si="4"/>
+        <v>0.35</v>
+      </c>
+      <c r="D45" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E45" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F45" s="17">
+        <f t="shared" si="4"/>
+        <v>5.7142857142857141E-2</v>
+      </c>
+      <c r="G45" s="18">
+        <f t="shared" si="5"/>
+        <v>0.40714285714285714</v>
+      </c>
+      <c r="H45" s="23">
+        <f>RANK(G45,$G$42:$G$51,0)+COUNTIF($G$42:G45,G45)-1</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="8" t="str">
+        <f t="shared" si="6"/>
+        <v>P10</v>
+      </c>
+      <c r="C46" s="17">
+        <f t="shared" si="4"/>
+        <v>0.35</v>
+      </c>
+      <c r="D46" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E46" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F46" s="17">
+        <f t="shared" si="4"/>
+        <v>2.8571428571428571E-2</v>
+      </c>
+      <c r="G46" s="18">
+        <f t="shared" si="5"/>
+        <v>0.37857142857142856</v>
+      </c>
+      <c r="H46" s="23">
+        <f>RANK(G46,$G$42:$G$51,0)+COUNTIF($G$42:G46,G46)-1</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="8" t="str">
+        <f t="shared" si="6"/>
+        <v>P5</v>
+      </c>
+      <c r="C47" s="17">
+        <f t="shared" si="4"/>
+        <v>0.23333333333333331</v>
+      </c>
+      <c r="D47" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E47" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F47" s="17">
+        <f t="shared" si="4"/>
+        <v>0.14285714285714288</v>
+      </c>
+      <c r="G47" s="18">
+        <f t="shared" si="5"/>
+        <v>0.37619047619047619</v>
+      </c>
+      <c r="H47" s="23">
+        <f>RANK(G47,$G$42:$G$51,0)+COUNTIF($G$42:G47,G47)-1</f>
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C43" s="17">
-        <f t="shared" si="3"/>
-        <v>8.7499999999999994E-2</v>
-      </c>
-      <c r="D43" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E43" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="F43" s="17">
-        <f t="shared" si="3"/>
-        <v>0.16666666666666669</v>
-      </c>
-      <c r="G43" s="18">
-        <f t="shared" si="4"/>
-        <v>0.25416666666666665</v>
-      </c>
-      <c r="H43" s="12">
+    <row r="48" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B48" s="8" t="str">
+        <f t="shared" si="6"/>
+        <v>P4</v>
+      </c>
+      <c r="C48" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="D48" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E48" s="17">
+        <f t="shared" si="4"/>
+        <v>0.15</v>
+      </c>
+      <c r="F48" s="17">
+        <f t="shared" si="4"/>
+        <v>0.17142857142857143</v>
+      </c>
+      <c r="G48" s="18">
         <f t="shared" si="5"/>
+        <v>0.3214285714285714</v>
+      </c>
+      <c r="H48" s="23">
+        <f>RANK(G48,$G$42:$G$51,0)+COUNTIF($G$42:G48,G48)-1</f>
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C44" s="17">
-        <f t="shared" si="3"/>
-        <v>0.17499999999999999</v>
-      </c>
-      <c r="D44" s="17">
-        <f t="shared" si="3"/>
-        <v>0.3</v>
-      </c>
-      <c r="E44" s="17">
-        <f t="shared" si="3"/>
-        <v>0.15</v>
-      </c>
-      <c r="F44" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G44" s="18">
-        <f t="shared" si="4"/>
-        <v>0.625</v>
-      </c>
-      <c r="H44" s="12">
+    <row r="49" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B49" s="8" t="str">
+        <f t="shared" si="6"/>
+        <v>P2</v>
+      </c>
+      <c r="C49" s="17">
+        <f t="shared" si="4"/>
+        <v>0.11666666666666665</v>
+      </c>
+      <c r="D49" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E49" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F49" s="17">
+        <f t="shared" si="4"/>
+        <v>0.14285714285714288</v>
+      </c>
+      <c r="G49" s="18">
         <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="45" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C45" s="17">
-        <f t="shared" si="3"/>
-        <v>0.35</v>
-      </c>
-      <c r="D45" s="17">
-        <f t="shared" si="3"/>
-        <v>0.15</v>
-      </c>
-      <c r="E45" s="17">
-        <f t="shared" si="3"/>
-        <v>0.15</v>
-      </c>
-      <c r="F45" s="17">
-        <f t="shared" si="3"/>
+        <v>0.25952380952380955</v>
+      </c>
+      <c r="H49" s="23">
+        <f>RANK(G49,$G$42:$G$51,0)+COUNTIF($G$42:G49,G49)-1</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B50" s="8" t="str">
+        <f t="shared" si="6"/>
+        <v>P7</v>
+      </c>
+      <c r="C50" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="D50" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E50" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F50" s="17">
+        <f t="shared" si="4"/>
         <v>0.2</v>
       </c>
-      <c r="G45" s="18">
-        <f t="shared" si="4"/>
-        <v>0.85000000000000009</v>
-      </c>
-      <c r="H45" s="12">
+      <c r="G50" s="18">
         <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C46" s="17">
-        <f t="shared" si="3"/>
-        <v>0.35</v>
-      </c>
-      <c r="D46" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E46" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="F46" s="17">
-        <f t="shared" si="3"/>
-        <v>0.16666666666666669</v>
-      </c>
-      <c r="G46" s="18">
-        <f t="shared" si="4"/>
-        <v>0.51666666666666661</v>
-      </c>
-      <c r="H46" s="12">
+        <v>0.2</v>
+      </c>
+      <c r="H50" s="23">
+        <f>RANK(G50,$G$42:$G$51,0)+COUNTIF($G$42:G50,G50)-1</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="8" t="str">
+        <f t="shared" si="6"/>
+        <v>P9</v>
+      </c>
+      <c r="C51" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="D51" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E51" s="17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F51" s="17">
+        <f t="shared" si="4"/>
+        <v>0.2</v>
+      </c>
+      <c r="G51" s="18">
         <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="47" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C47" s="17">
-        <f t="shared" si="3"/>
-        <v>0.35</v>
-      </c>
-      <c r="D47" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E47" s="17">
-        <f t="shared" si="3"/>
-        <v>0.15</v>
-      </c>
-      <c r="F47" s="17">
-        <f t="shared" si="3"/>
-        <v>0.16666666666666669</v>
-      </c>
-      <c r="G47" s="18">
-        <f t="shared" si="4"/>
-        <v>0.66666666666666674</v>
-      </c>
-      <c r="H47" s="12">
-        <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="48" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C48" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="D48" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E48" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="F48" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G48" s="18">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="H48" s="12">
-        <f t="shared" si="5"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="49" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C49" s="17">
-        <f t="shared" si="3"/>
-        <v>0.26249999999999996</v>
-      </c>
-      <c r="D49" s="17">
-        <f t="shared" si="3"/>
-        <v>0.3</v>
-      </c>
-      <c r="E49" s="17">
-        <f t="shared" si="3"/>
-        <v>0.15</v>
-      </c>
-      <c r="F49" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G49" s="18">
-        <f t="shared" si="4"/>
-        <v>0.71250000000000002</v>
-      </c>
-      <c r="H49" s="12">
-        <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="50" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C50" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="D50" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E50" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="F50" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G50" s="18">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="H50" s="12">
-        <f t="shared" si="5"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="51" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C51" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="D51" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E51" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="F51" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G51" s="18">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="H51" s="12">
-        <f t="shared" si="5"/>
+        <v>0.2</v>
+      </c>
+      <c r="H51" s="23">
+        <f>RANK(G51,$G$42:$G$51,0)+COUNTIF($G$42:G51,G51)-1</f>
         <v>10</v>
       </c>
     </row>
@@ -1690,141 +1787,141 @@
     </row>
     <row r="55" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B55" s="17">
-        <f t="shared" ref="B55:B64" si="6">G42</f>
-        <v>0.3833333333333333</v>
+        <f t="shared" ref="B55:B64" si="7">G42</f>
+        <v>0.91428571428571426</v>
       </c>
       <c r="C55" s="17" t="str">
-        <f t="shared" ref="C55:C64" si="7">B42</f>
-        <v>P9</v>
+        <f t="shared" ref="C55:C64" si="8">B42</f>
+        <v>P8</v>
       </c>
       <c r="D55" s="8">
-        <f t="shared" ref="D55:D64" si="8">H42</f>
-        <v>6</v>
+        <f t="shared" ref="D55:D64" si="9">H42</f>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B56" s="17">
-        <f t="shared" si="6"/>
-        <v>0.25416666666666665</v>
+        <f t="shared" si="7"/>
+        <v>0.68333333333333335</v>
       </c>
       <c r="C56" s="17" t="str">
-        <f t="shared" si="7"/>
-        <v>P8</v>
+        <f t="shared" si="8"/>
+        <v>P3</v>
       </c>
       <c r="D56" s="8">
-        <f t="shared" si="8"/>
-        <v>7</v>
+        <f t="shared" si="9"/>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B57" s="17">
-        <f t="shared" si="6"/>
-        <v>0.625</v>
+        <f t="shared" si="7"/>
+        <v>0.40952380952380951</v>
       </c>
       <c r="C57" s="17" t="str">
-        <f t="shared" si="7"/>
-        <v>P7</v>
+        <f t="shared" si="8"/>
+        <v>P6</v>
       </c>
       <c r="D57" s="8">
-        <f t="shared" si="8"/>
-        <v>4</v>
+        <f t="shared" si="9"/>
+        <v>3</v>
       </c>
     </row>
     <row r="58" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B58" s="17">
-        <f t="shared" si="6"/>
-        <v>0.85000000000000009</v>
+        <f t="shared" si="7"/>
+        <v>0.40714285714285714</v>
       </c>
       <c r="C58" s="17" t="str">
-        <f t="shared" si="7"/>
-        <v>P6</v>
+        <f t="shared" si="8"/>
+        <v>P10</v>
       </c>
       <c r="D58" s="8">
-        <f t="shared" si="8"/>
-        <v>1</v>
+        <f t="shared" si="9"/>
+        <v>4</v>
       </c>
     </row>
     <row r="59" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B59" s="17">
-        <f t="shared" si="6"/>
-        <v>0.51666666666666661</v>
+        <f t="shared" si="7"/>
+        <v>0.37857142857142856</v>
       </c>
       <c r="C59" s="17" t="str">
-        <f t="shared" si="7"/>
-        <v>P5</v>
+        <f t="shared" si="8"/>
+        <v>P10</v>
       </c>
       <c r="D59" s="8">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
     </row>
     <row r="60" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B60" s="17">
-        <f t="shared" si="6"/>
-        <v>0.66666666666666674</v>
+        <f t="shared" si="7"/>
+        <v>0.37619047619047619</v>
       </c>
       <c r="C60" s="17" t="str">
-        <f t="shared" si="7"/>
-        <v>P4</v>
+        <f t="shared" si="8"/>
+        <v>P5</v>
       </c>
       <c r="D60" s="8">
-        <f t="shared" si="8"/>
-        <v>3</v>
+        <f t="shared" si="9"/>
+        <v>6</v>
       </c>
     </row>
     <row r="61" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B61" s="17">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>0.3214285714285714</v>
       </c>
       <c r="C61" s="17" t="str">
-        <f t="shared" si="7"/>
-        <v>P3</v>
+        <f t="shared" si="8"/>
+        <v>P4</v>
       </c>
       <c r="D61" s="8">
-        <f t="shared" si="8"/>
-        <v>10</v>
+        <f t="shared" si="9"/>
+        <v>7</v>
       </c>
     </row>
     <row r="62" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B62" s="17">
-        <f t="shared" si="6"/>
-        <v>0.71250000000000002</v>
+        <f t="shared" si="7"/>
+        <v>0.25952380952380955</v>
       </c>
       <c r="C62" s="17" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>P2</v>
       </c>
       <c r="D62" s="8">
-        <f t="shared" si="8"/>
-        <v>2</v>
+        <f t="shared" si="9"/>
+        <v>8</v>
       </c>
     </row>
     <row r="63" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B63" s="17">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>0.2</v>
       </c>
       <c r="C63" s="17" t="str">
-        <f t="shared" si="7"/>
-        <v>P10</v>
+        <f t="shared" si="8"/>
+        <v>P7</v>
       </c>
       <c r="D63" s="8">
-        <f t="shared" si="8"/>
-        <v>10</v>
+        <f t="shared" si="9"/>
+        <v>9</v>
       </c>
     </row>
     <row r="64" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B64" s="17">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>0.2</v>
       </c>
       <c r="C64" s="17" t="str">
-        <f t="shared" si="7"/>
-        <v>P1</v>
+        <f t="shared" si="8"/>
+        <v>P9</v>
       </c>
       <c r="D64" s="8">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>10</v>
       </c>
     </row>
@@ -1884,17 +1981,20 @@
       <c r="A2">
         <v>1</v>
       </c>
+      <c r="B2" t="s">
+        <v>70</v>
+      </c>
       <c r="C2" t="s">
         <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="E2">
         <v>157600000</v>
       </c>
       <c r="F2" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="G2">
         <v>5</v>
@@ -1907,17 +2007,20 @@
       <c r="A3">
         <v>2</v>
       </c>
+      <c r="B3" t="s">
+        <v>70</v>
+      </c>
       <c r="C3" t="s">
         <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="E3">
         <v>383900000</v>
       </c>
       <c r="F3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G3">
         <v>5</v>
@@ -1930,17 +2033,20 @@
       <c r="A4">
         <v>3</v>
       </c>
+      <c r="B4" t="s">
+        <v>70</v>
+      </c>
       <c r="C4" t="s">
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>73</v>
       </c>
       <c r="E4">
         <v>285000000</v>
       </c>
       <c r="F4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G4">
         <v>8</v>
@@ -1953,17 +2059,20 @@
       <c r="A5">
         <v>4</v>
       </c>
+      <c r="B5" t="s">
+        <v>70</v>
+      </c>
       <c r="C5" t="s">
         <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E5">
         <v>606400000</v>
       </c>
       <c r="F5" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G5">
         <v>4</v>
@@ -1976,17 +2085,20 @@
       <c r="A6">
         <v>5</v>
       </c>
+      <c r="B6" t="s">
+        <v>70</v>
+      </c>
       <c r="C6" t="s">
         <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="E6">
         <v>274900000</v>
       </c>
       <c r="F6" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="G6">
         <v>5</v>
@@ -1999,17 +2111,20 @@
       <c r="A7">
         <v>6</v>
       </c>
+      <c r="B7" t="s">
+        <v>70</v>
+      </c>
       <c r="C7" t="s">
         <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E7">
         <v>352500000</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G7">
         <v>5</v>
@@ -2022,17 +2137,20 @@
       <c r="A8">
         <v>7</v>
       </c>
+      <c r="B8" t="s">
+        <v>70</v>
+      </c>
       <c r="C8" t="s">
         <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="E8">
         <v>749100000</v>
       </c>
       <c r="F8" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G8">
         <v>5</v>
@@ -2045,17 +2163,20 @@
       <c r="A9">
         <v>8</v>
       </c>
+      <c r="B9" t="s">
+        <v>70</v>
+      </c>
       <c r="C9" t="s">
         <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E9">
         <v>239600000</v>
       </c>
       <c r="F9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G9">
         <v>8</v>
@@ -2068,17 +2189,20 @@
       <c r="A10">
         <v>9</v>
       </c>
+      <c r="B10" t="s">
+        <v>70</v>
+      </c>
       <c r="C10" t="s">
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E10">
         <v>959900000</v>
       </c>
       <c r="F10" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="G10">
         <v>5</v>
@@ -2091,23 +2215,26 @@
       <c r="A11">
         <v>10</v>
       </c>
+      <c r="B11" t="s">
+        <v>70</v>
+      </c>
       <c r="C11" t="s">
         <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="E11">
-        <v>749100000</v>
+        <v>243100000</v>
       </c>
       <c r="F11" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="G11">
         <v>5</v>
       </c>
       <c r="H11">
-        <v>1993</v>
+        <v>1200</v>
       </c>
     </row>
   </sheetData>
@@ -2117,7 +2244,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C7D68FC-CBC7-4D03-8795-D9B86528E3D9}">
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
@@ -2144,28 +2271,28 @@
         <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="E1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="F1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="G1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="I1" t="s">
         <v>33</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="K1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="L1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -2176,7 +2303,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D2" t="s">
         <v>37</v>
@@ -2188,7 +2315,7 @@
         <v>2.4305555555555556E-2</v>
       </c>
       <c r="G2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="I2">
         <v>1</v>
@@ -2197,7 +2324,7 @@
         <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L2">
         <v>4</v>
@@ -2211,7 +2338,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
         <v>39</v>
@@ -2223,7 +2350,7 @@
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="G3" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I3">
         <v>2</v>
@@ -2232,7 +2359,7 @@
         <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L3">
         <v>3</v>
@@ -2246,7 +2373,7 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D4" t="s">
         <v>38</v>
@@ -2258,7 +2385,7 @@
         <v>1.0416666666666666E-2</v>
       </c>
       <c r="G4" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I4">
         <v>3</v>
@@ -2267,7 +2394,7 @@
         <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L4">
         <v>2</v>
@@ -2281,7 +2408,7 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D5" t="s">
         <v>40</v>
@@ -2293,7 +2420,7 @@
         <v>1.3888888888888888E-2</v>
       </c>
       <c r="G5" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I5">
         <v>4</v>
@@ -2302,7 +2429,7 @@
         <v>1</v>
       </c>
       <c r="K5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="L5">
         <v>1</v>
@@ -2372,7 +2499,7 @@
         <v>3</v>
       </c>
       <c r="K10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="L10">
         <v>4</v>
@@ -2386,7 +2513,7 @@
         <v>3</v>
       </c>
       <c r="K11" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="L11">
         <v>3</v>
@@ -2400,7 +2527,7 @@
         <v>3</v>
       </c>
       <c r="K12" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="L12">
         <v>2</v>
@@ -2414,7 +2541,7 @@
         <v>3</v>
       </c>
       <c r="K13" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="L13">
         <v>1</v>
@@ -2428,10 +2555,10 @@
         <v>4</v>
       </c>
       <c r="K14">
-        <v>1500</v>
+        <v>1193</v>
       </c>
       <c r="L14">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -2442,10 +2569,10 @@
         <v>4</v>
       </c>
       <c r="K15">
-        <v>1498</v>
+        <v>1198</v>
       </c>
       <c r="L15">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -2456,10 +2583,10 @@
         <v>4</v>
       </c>
       <c r="K16">
-        <v>1408</v>
+        <v>1199</v>
       </c>
       <c r="L16">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="9:12" x14ac:dyDescent="0.25">
@@ -2470,10 +2597,52 @@
         <v>4</v>
       </c>
       <c r="K17">
-        <v>1199</v>
+        <v>1408</v>
       </c>
       <c r="L17">
-        <v>1</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="I18">
+        <v>17</v>
+      </c>
+      <c r="J18">
+        <v>4</v>
+      </c>
+      <c r="K18">
+        <v>1496</v>
+      </c>
+      <c r="L18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="I19">
+        <v>18</v>
+      </c>
+      <c r="J19">
+        <v>4</v>
+      </c>
+      <c r="K19">
+        <v>1498</v>
+      </c>
+      <c r="L19">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="I20">
+        <v>19</v>
+      </c>
+      <c r="J20">
+        <v>4</v>
+      </c>
+      <c r="K20">
+        <v>1500</v>
+      </c>
+      <c r="L20">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>